<commit_message>
Actualizacion datos REM 2026-09-29 16:25 (orquestador)
</commit_message>
<xml_diff>
--- a/output/REM_2024_P1_SECCION_D_GESTANTES.xlsx
+++ b/output/REM_2024_P1_SECCION_D_GESTANTES.xlsx
@@ -145,7 +145,7 @@
     <t>Posta de Salud Rural Las Canteras</t>
   </si>
   <si>
-    <t>Centro Comunitario de Salud Familiar Dr. José Symón Ojeda</t>
+    <t>CECOSF Haydeé Sepúlveda</t>
   </si>
   <si>
     <t>Posta de Salud Rural Chacabuco (Colina)</t>
@@ -223,7 +223,7 @@
     <t>Centro Comunitario de Salud Familiar Batuco</t>
   </si>
   <si>
-    <t>Hospital de Til Til</t>
+    <t>Hospital Comunitario de Til Til</t>
   </si>
   <si>
     <t>Centro de Salud Familiar Apoquindo</t>
@@ -421,7 +421,7 @@
     <t>Centro Comunitario de Salud Familiar Padre Demetrio Bravo</t>
   </si>
   <si>
-    <t>Centro Comunitario de Salud Familiar Lo Chacón</t>
+    <t>CECOSF Wilma Yoli Gomez Conejera</t>
   </si>
   <si>
     <t>Centro de Salud Familiar La Islita</t>
@@ -481,7 +481,7 @@
     <t>Centro de Salud Familiar Santa Anselma</t>
   </si>
   <si>
-    <t>Centro de Salud Familiar Maipo</t>
+    <t>Centro de Salud Familiar Dragica Ciudad Pap</t>
   </si>
   <si>
     <t>Centro de Salud Familiar Dr. Miguel Ángel Solar (ex CESFAM Paine)</t>
@@ -1045,7 +1045,7 @@
     <t>Estación Central</t>
   </si>
   <si>
-    <t>Servicio de Salud Metropolitano Sur Oriente</t>
+    <t>Servicio de Salud Metropolitano Sur - Oriente</t>
   </si>
   <si>
     <t>Servicio de Salud Metropolitano Central</t>

</xml_diff>